<commit_message>
add of new element
</commit_message>
<xml_diff>
--- a/boxes.xlsx
+++ b/boxes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fofr6825\Documents\MATLAB\Adaptive-Palletizing\Adaptive-Palletizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72114BA1-9E30-45FF-B05A-5A2C8D1141E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ACD1108-3C98-4868-B68A-97BAB34C3E18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1D3690FE-5D9A-45E6-8524-1FA8AE5358A6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>id</t>
   </si>
@@ -63,12 +63,6 @@
   </si>
   <si>
     <t>pickZ</t>
-  </si>
-  <si>
-    <t>0.2</t>
-  </si>
-  <si>
-    <t>0.3</t>
   </si>
 </sst>
 </file>
@@ -502,14 +496,14 @@
       <c r="D2" s="2">
         <v>0.2</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>8</v>
+      <c r="E2" s="2">
+        <v>0.2</v>
       </c>
       <c r="F2" s="2">
         <v>-0.65</v>
       </c>
       <c r="G2" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H2" s="2">
         <v>0.6</v>
@@ -528,14 +522,14 @@
       <c r="D3" s="2">
         <v>0.2</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>8</v>
+      <c r="E3" s="2">
+        <v>0.2</v>
       </c>
       <c r="F3" s="2">
         <v>-0.65</v>
       </c>
       <c r="G3" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H3" s="2">
         <v>0.6</v>
@@ -554,14 +548,14 @@
       <c r="D4" s="2">
         <v>0.2</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>8</v>
+      <c r="E4" s="2">
+        <v>0.2</v>
       </c>
       <c r="F4" s="2">
         <v>-0.65</v>
       </c>
       <c r="G4" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H4" s="2">
         <v>0.6</v>
@@ -580,14 +574,14 @@
       <c r="D5" s="2">
         <v>0.2</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>8</v>
+      <c r="E5" s="2">
+        <v>0.2</v>
       </c>
       <c r="F5" s="2">
         <v>-0.65</v>
       </c>
       <c r="G5" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H5" s="2">
         <v>0.6</v>
@@ -606,14 +600,14 @@
       <c r="D6" s="2">
         <v>0.2</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>8</v>
+      <c r="E6" s="2">
+        <v>0.2</v>
       </c>
       <c r="F6" s="2">
         <v>-0.65</v>
       </c>
       <c r="G6" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H6" s="2">
         <v>0.6</v>
@@ -632,14 +626,14 @@
       <c r="D7" s="2">
         <v>0.2</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>8</v>
+      <c r="E7" s="2">
+        <v>0.2</v>
       </c>
       <c r="F7" s="2">
         <v>-0.65</v>
       </c>
       <c r="G7" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H7" s="2">
         <v>0.6</v>
@@ -658,14 +652,14 @@
       <c r="D8" s="2">
         <v>0.2</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>8</v>
+      <c r="E8" s="2">
+        <v>0.2</v>
       </c>
       <c r="F8" s="2">
         <v>-0.65</v>
       </c>
       <c r="G8" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H8" s="2">
         <v>0.6</v>
@@ -684,14 +678,14 @@
       <c r="D9" s="2">
         <v>0.2</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>8</v>
+      <c r="E9" s="2">
+        <v>0.2</v>
       </c>
       <c r="F9" s="2">
         <v>-0.65</v>
       </c>
       <c r="G9" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H9" s="2">
         <v>0.6</v>
@@ -710,14 +704,14 @@
       <c r="D10" s="2">
         <v>0.2</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>8</v>
+      <c r="E10" s="2">
+        <v>0.2</v>
       </c>
       <c r="F10" s="2">
         <v>-0.65</v>
       </c>
       <c r="G10" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H10" s="2">
         <v>0.6</v>
@@ -736,14 +730,14 @@
       <c r="D11" s="2">
         <v>0.2</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>8</v>
+      <c r="E11" s="2">
+        <v>0.2</v>
       </c>
       <c r="F11" s="2">
         <v>-0.65</v>
       </c>
       <c r="G11" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H11" s="2">
         <v>0.6</v>
@@ -762,14 +756,14 @@
       <c r="D12" s="2">
         <v>0.2</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>8</v>
+      <c r="E12" s="2">
+        <v>0.2</v>
       </c>
       <c r="F12" s="2">
         <v>-0.65</v>
       </c>
       <c r="G12" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H12" s="2">
         <v>0.6</v>
@@ -788,14 +782,14 @@
       <c r="D13" s="2">
         <v>0.2</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>8</v>
+      <c r="E13" s="2">
+        <v>0.2</v>
       </c>
       <c r="F13" s="2">
         <v>-0.65</v>
       </c>
       <c r="G13" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H13" s="2">
         <v>0.6</v>
@@ -814,14 +808,14 @@
       <c r="D14" s="2">
         <v>0.2</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>8</v>
+      <c r="E14" s="2">
+        <v>0.2</v>
       </c>
       <c r="F14" s="2">
         <v>-0.65</v>
       </c>
       <c r="G14" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H14" s="2">
         <v>0.6</v>
@@ -840,14 +834,14 @@
       <c r="D15" s="2">
         <v>0.2</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>8</v>
+      <c r="E15" s="2">
+        <v>0.2</v>
       </c>
       <c r="F15" s="2">
         <v>-0.65</v>
       </c>
       <c r="G15" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H15" s="2">
         <v>0.6</v>
@@ -866,14 +860,14 @@
       <c r="D16" s="2">
         <v>0.2</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>8</v>
+      <c r="E16" s="2">
+        <v>0.2</v>
       </c>
       <c r="F16" s="2">
         <v>-0.65</v>
       </c>
       <c r="G16" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H16" s="2">
         <v>0.6</v>
@@ -892,14 +886,14 @@
       <c r="D17" s="2">
         <v>0.2</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>8</v>
+      <c r="E17" s="2">
+        <v>0.2</v>
       </c>
       <c r="F17" s="2">
         <v>-0.65</v>
       </c>
       <c r="G17" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H17" s="2">
         <v>0.6</v>
@@ -918,14 +912,14 @@
       <c r="D18" s="2">
         <v>0.2</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>8</v>
+      <c r="E18" s="2">
+        <v>0.2</v>
       </c>
       <c r="F18" s="2">
         <v>-0.65</v>
       </c>
       <c r="G18" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H18" s="2">
         <v>0.6</v>
@@ -944,14 +938,14 @@
       <c r="D19" s="2">
         <v>0.2</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>8</v>
+      <c r="E19" s="2">
+        <v>0.2</v>
       </c>
       <c r="F19" s="2">
         <v>-0.65</v>
       </c>
       <c r="G19" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H19" s="2">
         <v>0.6</v>
@@ -970,14 +964,14 @@
       <c r="D20" s="2">
         <v>0.2</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>8</v>
+      <c r="E20" s="2">
+        <v>0.2</v>
       </c>
       <c r="F20" s="2">
         <v>-0.65</v>
       </c>
       <c r="G20" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H20" s="2">
         <v>0.6</v>
@@ -996,14 +990,14 @@
       <c r="D21" s="2">
         <v>0.2</v>
       </c>
-      <c r="E21" s="2" t="s">
-        <v>8</v>
+      <c r="E21" s="2">
+        <v>0.2</v>
       </c>
       <c r="F21" s="2">
         <v>-0.65</v>
       </c>
       <c r="G21" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H21" s="2">
         <v>0.6</v>
@@ -1022,14 +1016,14 @@
       <c r="D22" s="2">
         <v>0.2</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>8</v>
+      <c r="E22" s="2">
+        <v>0.2</v>
       </c>
       <c r="F22" s="2">
         <v>-0.65</v>
       </c>
       <c r="G22" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H22" s="2">
         <v>0.6</v>
@@ -1048,14 +1042,14 @@
       <c r="D23" s="2">
         <v>0.2</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>8</v>
+      <c r="E23" s="2">
+        <v>0.2</v>
       </c>
       <c r="F23" s="2">
         <v>-0.65</v>
       </c>
       <c r="G23" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H23" s="2">
         <v>0.6</v>
@@ -1074,14 +1068,14 @@
       <c r="D24" s="2">
         <v>0.2</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>8</v>
+      <c r="E24" s="2">
+        <v>0.2</v>
       </c>
       <c r="F24" s="2">
         <v>-0.65</v>
       </c>
       <c r="G24" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H24" s="2">
         <v>0.6</v>
@@ -1100,14 +1094,14 @@
       <c r="D25" s="2">
         <v>0.2</v>
       </c>
-      <c r="E25" s="2" t="s">
-        <v>8</v>
+      <c r="E25" s="2">
+        <v>0.2</v>
       </c>
       <c r="F25" s="2">
         <v>-0.65</v>
       </c>
       <c r="G25" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H25" s="2">
         <v>0.6</v>
@@ -1126,14 +1120,14 @@
       <c r="D26" s="2">
         <v>0.2</v>
       </c>
-      <c r="E26" s="2" t="s">
-        <v>8</v>
+      <c r="E26" s="2">
+        <v>0.2</v>
       </c>
       <c r="F26" s="2">
         <v>-0.65</v>
       </c>
       <c r="G26" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H26" s="2">
         <v>0.6</v>
@@ -1152,14 +1146,14 @@
       <c r="D27" s="2">
         <v>0.2</v>
       </c>
-      <c r="E27" s="2" t="s">
-        <v>8</v>
+      <c r="E27" s="2">
+        <v>0.2</v>
       </c>
       <c r="F27" s="2">
         <v>-0.65</v>
       </c>
       <c r="G27" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H27" s="2">
         <v>0.6</v>
@@ -1178,14 +1172,14 @@
       <c r="D28" s="2">
         <v>0.2</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>8</v>
+      <c r="E28" s="2">
+        <v>0.2</v>
       </c>
       <c r="F28" s="2">
         <v>-0.65</v>
       </c>
       <c r="G28" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H28" s="2">
         <v>0.6</v>
@@ -1204,14 +1198,14 @@
       <c r="D29" s="2">
         <v>0.2</v>
       </c>
-      <c r="E29" s="2" t="s">
-        <v>8</v>
+      <c r="E29" s="2">
+        <v>0.2</v>
       </c>
       <c r="F29" s="2">
         <v>-0.65</v>
       </c>
       <c r="G29" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H29" s="2">
         <v>0.6</v>
@@ -1230,14 +1224,14 @@
       <c r="D30" s="2">
         <v>0.2</v>
       </c>
-      <c r="E30" s="2" t="s">
-        <v>8</v>
+      <c r="E30" s="2">
+        <v>0.2</v>
       </c>
       <c r="F30" s="2">
         <v>-0.65</v>
       </c>
       <c r="G30" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H30" s="2">
         <v>0.6</v>
@@ -1256,14 +1250,14 @@
       <c r="D31" s="2">
         <v>0.2</v>
       </c>
-      <c r="E31" s="2" t="s">
-        <v>9</v>
+      <c r="E31" s="2">
+        <v>0.2</v>
       </c>
       <c r="F31" s="2">
         <v>-0.65</v>
       </c>
       <c r="G31" s="2">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="H31" s="2">
         <v>0.6</v>

</xml_diff>